<commit_message>
Laminas comunales de Ingresos y Demografia regeneradas
Lote 2 de 6.
El commit original (b1bed81b) cambiaba 13.973 archivos y 2,40 GB de objetos
nuevos en una sola pieza. GitHub rechaza los push sobre 2 GB por HTTPS, y SSH
esta bloqueado en esta red, asi que ese commit no podia subir nunca: el HTTP 500
no era un error transitorio sino el limite. Se trocea por dimension, que es un
corte con sentido, no alfabetico.
</commit_message>
<xml_diff>
--- a/output/graficos_dimensiones/comunal_i_ingr_a_2018_antofagasta.xlsx
+++ b/output/graficos_dimensiones/comunal_i_ingr_a_2018_antofagasta.xlsx
@@ -51,15 +51,15 @@
     <t xml:space="preserve">San Pedro de Atacama</t>
   </si>
   <si>
+    <t xml:space="preserve">Ollagüe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sierra Gorda</t>
+  </si>
+  <si>
     <t xml:space="preserve">María Elena</t>
   </si>
   <si>
-    <t xml:space="preserve">Sierra Gorda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ollagüe</t>
-  </si>
-  <si>
     <t xml:space="preserve">Campo</t>
   </si>
   <si>
@@ -69,7 +69,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-06 20:06</t>
+    <t xml:space="preserve">2026-09-09 22:59</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -601,7 +601,7 @@
         <v>11</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2302</v>
+        <v>2202</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -627,7 +627,7 @@
         <v>13</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>2202</v>
+        <v>2302</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>

</xml_diff>